<commit_message>
feat: filter out non-declared areas in thermal parser and update tests
- Added `_filter_non_declared_areas` method to exclude nodes outside the RTE study perimeter.
- Integrated the new filter into the thermal parser pipeline.
- Updated expected output Excel files for 2030 and 2035 to reflect filtering changes.
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/specific_2030.xlsx
+++ b/tests/antares/resources/expected_output_files/specific_2030.xlsx
@@ -888,13 +888,13 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1.290243902439024</v>
+        <v>1.940650406504065</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>0.4705734089477001</v>
+        <v>0.4737327188940092</v>
       </c>
       <c r="I4" t="n">
         <v>0.08</v>
@@ -917,7 +917,7 @@
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R4" t="n">
         <v>0.08</v>
@@ -956,13 +956,13 @@
         <v>0.08</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.02225274725274726</v>
+        <v>0.02225274725274725</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.02225274725274726</v>
+        <v>0.02225274725274725</v>
       </c>
       <c r="AF4" t="n">
-        <v>0.02225274725274726</v>
+        <v>0.02225274725274725</v>
       </c>
       <c r="AG4" t="n">
         <v>0.1254098360655738</v>
@@ -983,13 +983,13 @@
         <v>0.1254098360655738</v>
       </c>
       <c r="AM4" t="n">
-        <v>0.02225274725274726</v>
+        <v>0.02225274725274725</v>
       </c>
       <c r="AN4" t="n">
-        <v>0.02225274725274726</v>
+        <v>0.02225274725274725</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.02225274725274726</v>
+        <v>0.02225274725274725</v>
       </c>
     </row>
     <row r="5">
@@ -1126,13 +1126,13 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>1.468413098236776</v>
+        <v>1.764836272040303</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0.58</v>
+        <v>0.5799999999999998</v>
       </c>
       <c r="I6" t="n">
         <v>0.05</v>
@@ -1155,7 +1155,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R6" t="n">
         <v>0.05</v>
@@ -2316,13 +2316,13 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="n">
-        <v>0.6116270597305503</v>
+        <v>0.7510384754125735</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0.420622091129367</v>
+        <v>0.4217078285682363</v>
       </c>
       <c r="I16" t="n">
         <v>0.08000000000000002</v>
@@ -2345,7 +2345,7 @@
         <v>1</v>
       </c>
       <c r="Q16" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="R16" t="n">
         <v>0.08000000000000002</v>
@@ -2792,7 +2792,7 @@
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="n">
-        <v>0.6875</v>
+        <v>1.375</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -2821,7 +2821,7 @@
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R20" t="n">
         <v>0.05</v>
@@ -2911,16 +2911,16 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="n">
-        <v>0.7485714285714286</v>
+        <v>1.624761904761905</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>0.4569482288828338</v>
+        <v>0.3998729351969504</v>
       </c>
       <c r="I21" t="n">
-        <v>0.06716621253405994</v>
+        <v>0.07401524777636595</v>
       </c>
       <c r="J21" t="n">
         <v>1</v>
@@ -2929,7 +2929,7 @@
         <v>27</v>
       </c>
       <c r="L21" t="n">
-        <v>0.06416893732970028</v>
+        <v>0.02992376111817027</v>
       </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
@@ -2940,79 +2940,79 @@
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R21" t="n">
-        <v>0.06716621253405994</v>
+        <v>0.07401524777636595</v>
       </c>
       <c r="S21" t="n">
-        <v>0.06716621253405994</v>
+        <v>0.07401524777636595</v>
       </c>
       <c r="T21" t="n">
-        <v>0.06716621253405994</v>
+        <v>0.07401524777636595</v>
       </c>
       <c r="U21" t="n">
-        <v>0.06716621253405994</v>
+        <v>0.07401524777636595</v>
       </c>
       <c r="V21" t="n">
-        <v>0.06716621253405994</v>
+        <v>0.07401524777636595</v>
       </c>
       <c r="W21" t="n">
-        <v>0.06716621253405994</v>
+        <v>0.07401524777636595</v>
       </c>
       <c r="X21" t="n">
-        <v>0.06716621253405994</v>
+        <v>0.07401524777636595</v>
       </c>
       <c r="Y21" t="n">
-        <v>0.06716621253405994</v>
+        <v>0.07401524777636595</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.06716621253405994</v>
+        <v>0.07401524777636595</v>
       </c>
       <c r="AA21" t="n">
-        <v>0.06716621253405994</v>
+        <v>0.07401524777636595</v>
       </c>
       <c r="AB21" t="n">
-        <v>0.06716621253405994</v>
+        <v>0.07401524777636595</v>
       </c>
       <c r="AC21" t="n">
-        <v>0.06716621253405994</v>
+        <v>0.07401524777636595</v>
       </c>
       <c r="AD21" t="n">
-        <v>0.009519567625834656</v>
+        <v>0.004439239286761524</v>
       </c>
       <c r="AE21" t="n">
-        <v>0.009519567625834656</v>
+        <v>0.004439239286761524</v>
       </c>
       <c r="AF21" t="n">
-        <v>0.009519567625834656</v>
+        <v>0.004439239286761524</v>
       </c>
       <c r="AG21" t="n">
-        <v>0.1380734354759459</v>
+        <v>0.1431260024579749</v>
       </c>
       <c r="AH21" t="n">
-        <v>0.1380734354759459</v>
+        <v>0.1431260024579749</v>
       </c>
       <c r="AI21" t="n">
-        <v>0.1380734354759459</v>
+        <v>0.1431260024579749</v>
       </c>
       <c r="AJ21" t="n">
-        <v>0.1380734354759459</v>
+        <v>0.1431260024579749</v>
       </c>
       <c r="AK21" t="n">
-        <v>0.1380734354759459</v>
+        <v>0.1431260024579749</v>
       </c>
       <c r="AL21" t="n">
-        <v>0.1380734354759459</v>
+        <v>0.1431260024579749</v>
       </c>
       <c r="AM21" t="n">
-        <v>0.009519567625834656</v>
+        <v>0.004439239286761524</v>
       </c>
       <c r="AN21" t="n">
-        <v>0.009519567625834656</v>
+        <v>0.004439239286761524</v>
       </c>
       <c r="AO21" t="n">
-        <v>0.009519567625834656</v>
+        <v>0.004439239286761524</v>
       </c>
     </row>
     <row r="22">
@@ -4101,7 +4101,7 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="n">
-        <v>0.5121478270788182</v>
+        <v>1.536443481236455</v>
       </c>
       <c r="G31" t="n">
         <v>0</v>
@@ -4130,7 +4130,7 @@
         <v>1</v>
       </c>
       <c r="Q31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R31" t="n">
         <v>0.05</v>
@@ -4169,13 +4169,13 @@
         <v>0.05</v>
       </c>
       <c r="AD31" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AE31" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AF31" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AG31" t="n">
         <v>0.1254098360655738</v>
@@ -4196,13 +4196,13 @@
         <v>0.1254098360655738</v>
       </c>
       <c r="AM31" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AN31" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AO31" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
     </row>
     <row r="32">
@@ -4220,7 +4220,7 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
-        <v>1.354243542435424</v>
+        <v>2.708487084870849</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
@@ -4249,7 +4249,7 @@
         <v>1</v>
       </c>
       <c r="Q32" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R32" t="n">
         <v>0.098</v>
@@ -4339,7 +4339,7 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="n">
-        <v>0.9344262295081968</v>
+        <v>1.401639344262295</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
@@ -4368,7 +4368,7 @@
         <v>1</v>
       </c>
       <c r="Q33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R33" t="n">
         <v>0.168</v>
@@ -4407,13 +4407,13 @@
         <v>0.168</v>
       </c>
       <c r="AD33" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AE33" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AF33" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AG33" t="n">
         <v>0.1254098360655738</v>
@@ -4434,13 +4434,13 @@
         <v>0.1254098360655738</v>
       </c>
       <c r="AM33" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AN33" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AO33" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
     </row>
     <row r="34">
@@ -4458,7 +4458,7 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="n">
-        <v>0.4017216642754661</v>
+        <v>0.8034433285509323</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
@@ -4487,7 +4487,7 @@
         <v>1</v>
       </c>
       <c r="Q34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R34" t="n">
         <v>0.08</v>
@@ -4577,7 +4577,7 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="n">
-        <v>1.693251533742331</v>
+        <v>5.079754601226994</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -4606,7 +4606,7 @@
         <v>0</v>
       </c>
       <c r="Q35" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="R35" t="n">
         <v>0.11</v>
@@ -4696,7 +4696,7 @@
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="n">
-        <v>0.2133333333333333</v>
+        <v>0.4266666666666667</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
@@ -4725,7 +4725,7 @@
         <v>1</v>
       </c>
       <c r="Q36" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R36" t="n">
         <v>0.033</v>
@@ -4934,13 +4934,13 @@
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="n">
-        <v>1.047092783505155</v>
+        <v>1.050639175257732</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>0.6</v>
+        <v>0.5999999999999999</v>
       </c>
       <c r="I38" t="n">
         <v>0.04999999999999999</v>
@@ -4963,7 +4963,7 @@
         <v>0</v>
       </c>
       <c r="Q38" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R38" t="n">
         <v>0.04999999999999999</v>
@@ -5172,13 +5172,13 @@
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="n">
-        <v>0.9364548494983277</v>
+        <v>1.438127090301003</v>
       </c>
       <c r="G40" t="n">
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>0.5599999999999999</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I40" t="n">
         <v>0.05</v>
@@ -5201,7 +5201,7 @@
         <v>0</v>
       </c>
       <c r="Q40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R40" t="n">
         <v>0.05</v>
@@ -5410,22 +5410,22 @@
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="n">
-        <v>1.014348296497069</v>
+        <v>1.161247190572593</v>
       </c>
       <c r="G42" t="n">
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>0.3500000000000001</v>
+        <v>0.3499999999999999</v>
       </c>
       <c r="I42" t="n">
-        <v>0.1</v>
+        <v>0.09999999999999999</v>
       </c>
       <c r="J42" t="n">
         <v>1</v>
       </c>
       <c r="K42" t="n">
-        <v>27.00000000000001</v>
+        <v>27</v>
       </c>
       <c r="L42" t="n">
         <v>0.15</v>
@@ -5439,52 +5439,52 @@
         <v>1</v>
       </c>
       <c r="Q42" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R42" t="n">
-        <v>0.1</v>
+        <v>0.09999999999999999</v>
       </c>
       <c r="S42" t="n">
-        <v>0.1</v>
+        <v>0.09999999999999999</v>
       </c>
       <c r="T42" t="n">
-        <v>0.1</v>
+        <v>0.09999999999999999</v>
       </c>
       <c r="U42" t="n">
-        <v>0.1</v>
+        <v>0.09999999999999999</v>
       </c>
       <c r="V42" t="n">
-        <v>0.1</v>
+        <v>0.09999999999999999</v>
       </c>
       <c r="W42" t="n">
-        <v>0.1</v>
+        <v>0.09999999999999999</v>
       </c>
       <c r="X42" t="n">
-        <v>0.1</v>
+        <v>0.09999999999999999</v>
       </c>
       <c r="Y42" t="n">
-        <v>0.1</v>
+        <v>0.09999999999999999</v>
       </c>
       <c r="Z42" t="n">
-        <v>0.1</v>
+        <v>0.09999999999999999</v>
       </c>
       <c r="AA42" t="n">
-        <v>0.1</v>
+        <v>0.09999999999999999</v>
       </c>
       <c r="AB42" t="n">
-        <v>0.1</v>
+        <v>0.09999999999999999</v>
       </c>
       <c r="AC42" t="n">
-        <v>0.1</v>
+        <v>0.09999999999999999</v>
       </c>
       <c r="AD42" t="n">
-        <v>0.02225274725274726</v>
+        <v>0.02225274725274724</v>
       </c>
       <c r="AE42" t="n">
-        <v>0.02225274725274726</v>
+        <v>0.02225274725274724</v>
       </c>
       <c r="AF42" t="n">
-        <v>0.02225274725274726</v>
+        <v>0.02225274725274724</v>
       </c>
       <c r="AG42" t="n">
         <v>0.1254098360655738</v>
@@ -5505,13 +5505,13 @@
         <v>0.1254098360655738</v>
       </c>
       <c r="AM42" t="n">
-        <v>0.02225274725274726</v>
+        <v>0.02225274725274724</v>
       </c>
       <c r="AN42" t="n">
-        <v>0.02225274725274726</v>
+        <v>0.02225274725274724</v>
       </c>
       <c r="AO42" t="n">
-        <v>0.02225274725274726</v>
+        <v>0.02225274725274724</v>
       </c>
     </row>
     <row r="43">
@@ -5886,22 +5886,22 @@
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="n">
-        <v>1.986545454545454</v>
+        <v>2.011358288770054</v>
       </c>
       <c r="G46" t="n">
         <v>0</v>
       </c>
       <c r="H46" t="n">
-        <v>0.6</v>
+        <v>0.6000000000000001</v>
       </c>
       <c r="I46" t="n">
         <v>0.04730000000000002</v>
       </c>
       <c r="J46" t="n">
-        <v>3.67</v>
+        <v>3.670000000000001</v>
       </c>
       <c r="K46" t="n">
-        <v>70</v>
+        <v>70.00000000000001</v>
       </c>
       <c r="L46" t="n">
         <v>0.4600000000000001</v>
@@ -5915,7 +5915,7 @@
         <v>0</v>
       </c>
       <c r="Q46" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="R46" t="n">
         <v>0.04730000000000002</v>
@@ -6124,19 +6124,19 @@
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="n">
-        <v>1.611757105943152</v>
+        <v>1.642764857881137</v>
       </c>
       <c r="G48" t="n">
         <v>0</v>
       </c>
       <c r="H48" t="n">
-        <v>0.4920137404772082</v>
+        <v>0.4912861197110423</v>
       </c>
       <c r="I48" t="n">
         <v>0.0473</v>
       </c>
       <c r="J48" t="n">
-        <v>3.669999999999999</v>
+        <v>3.67</v>
       </c>
       <c r="K48" t="n">
         <v>70</v>
@@ -6153,7 +6153,7 @@
         <v>0</v>
       </c>
       <c r="Q48" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="R48" t="n">
         <v>0.0473</v>
@@ -6243,13 +6243,13 @@
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="n">
-        <v>4.4699</v>
+        <v>5.452000000000001</v>
       </c>
       <c r="G49" t="n">
         <v>0</v>
       </c>
       <c r="H49" t="n">
-        <v>0.5499999999999999</v>
+        <v>0.55</v>
       </c>
       <c r="I49" t="n">
         <v>0.04729999999999999</v>
@@ -6272,7 +6272,7 @@
         <v>0</v>
       </c>
       <c r="Q49" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="R49" t="n">
         <v>0.04729999999999999</v>
@@ -6362,7 +6362,7 @@
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="n">
-        <v>7.42689497716895</v>
+        <v>8.390182648401828</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
@@ -6371,7 +6371,7 @@
         <v>0.59</v>
       </c>
       <c r="I50" t="n">
-        <v>0.04729999999999999</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="J50" t="n">
         <v>3.67</v>
@@ -6380,7 +6380,7 @@
         <v>70</v>
       </c>
       <c r="L50" t="n">
-        <v>0.46</v>
+        <v>0.4600000000000001</v>
       </c>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
@@ -6391,52 +6391,52 @@
         <v>0</v>
       </c>
       <c r="Q50" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="R50" t="n">
-        <v>0.04729999999999999</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="S50" t="n">
-        <v>0.04729999999999999</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="T50" t="n">
-        <v>0.04729999999999999</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="U50" t="n">
-        <v>0.04729999999999999</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="V50" t="n">
-        <v>0.04729999999999999</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="W50" t="n">
-        <v>0.04729999999999999</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="X50" t="n">
-        <v>0.04729999999999999</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="Y50" t="n">
-        <v>0.04729999999999999</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="Z50" t="n">
-        <v>0.04729999999999999</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="AA50" t="n">
-        <v>0.04729999999999999</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="AB50" t="n">
-        <v>0.04729999999999999</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="AC50" t="n">
-        <v>0.04729999999999999</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="AD50" t="n">
-        <v>0.1769230769230769</v>
+        <v>0.176923076923077</v>
       </c>
       <c r="AE50" t="n">
-        <v>0.1769230769230769</v>
+        <v>0.176923076923077</v>
       </c>
       <c r="AF50" t="n">
-        <v>0.1769230769230769</v>
+        <v>0.176923076923077</v>
       </c>
       <c r="AG50" t="n">
         <v>0.2065573770491803</v>
@@ -6457,13 +6457,13 @@
         <v>0.2065573770491803</v>
       </c>
       <c r="AM50" t="n">
-        <v>0.1769230769230769</v>
+        <v>0.176923076923077</v>
       </c>
       <c r="AN50" t="n">
-        <v>0.1769230769230769</v>
+        <v>0.176923076923077</v>
       </c>
       <c r="AO50" t="n">
-        <v>0.1769230769230769</v>
+        <v>0.176923076923077</v>
       </c>
     </row>
     <row r="51">
@@ -6481,25 +6481,25 @@
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="n">
-        <v>1.86661153262769</v>
+        <v>3.135324480069333</v>
       </c>
       <c r="G51" t="n">
         <v>0</v>
       </c>
       <c r="H51" t="n">
-        <v>0.3861333744542214</v>
+        <v>0.3739424708652774</v>
       </c>
       <c r="I51" t="n">
-        <v>0.05231263231947191</v>
+        <v>0.06530650324021327</v>
       </c>
       <c r="J51" t="n">
-        <v>3.260711672997248</v>
+        <v>2.19974423084497</v>
       </c>
       <c r="K51" t="n">
-        <v>63.40846514564856</v>
+        <v>46.32172356791526</v>
       </c>
       <c r="L51" t="n">
-        <v>0.4124796324453734</v>
+        <v>0.2892961466524123</v>
       </c>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr"/>
@@ -6510,79 +6510,79 @@
         <v>1</v>
       </c>
       <c r="Q51" t="n">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="R51" t="n">
-        <v>0.05231263231947191</v>
+        <v>0.06530650324021327</v>
       </c>
       <c r="S51" t="n">
-        <v>0.05231263231947191</v>
+        <v>0.06530650324021327</v>
       </c>
       <c r="T51" t="n">
-        <v>0.05231263231947191</v>
+        <v>0.06530650324021327</v>
       </c>
       <c r="U51" t="n">
-        <v>0.05231263231947191</v>
+        <v>0.06530650324021327</v>
       </c>
       <c r="V51" t="n">
-        <v>0.05231263231947191</v>
+        <v>0.06530650324021327</v>
       </c>
       <c r="W51" t="n">
-        <v>0.05231263231947191</v>
+        <v>0.06530650324021327</v>
       </c>
       <c r="X51" t="n">
-        <v>0.05231263231947191</v>
+        <v>0.06530650324021327</v>
       </c>
       <c r="Y51" t="n">
-        <v>0.05231263231947191</v>
+        <v>0.06530650324021327</v>
       </c>
       <c r="Z51" t="n">
-        <v>0.05231263231947191</v>
+        <v>0.06530650324021327</v>
       </c>
       <c r="AA51" t="n">
-        <v>0.05231263231947191</v>
+        <v>0.06530650324021327</v>
       </c>
       <c r="AB51" t="n">
-        <v>0.05231263231947191</v>
+        <v>0.06530650324021327</v>
       </c>
       <c r="AC51" t="n">
-        <v>0.05231263231947191</v>
+        <v>0.06530650324021327</v>
       </c>
       <c r="AD51" t="n">
-        <v>0.1437071450395735</v>
+        <v>0.07363019854118745</v>
       </c>
       <c r="AE51" t="n">
-        <v>0.1437071450395735</v>
+        <v>0.07363019854118745</v>
       </c>
       <c r="AF51" t="n">
-        <v>0.1437071450395735</v>
+        <v>0.07363019854118745</v>
       </c>
       <c r="AG51" t="n">
-        <v>0.2035724849641867</v>
+        <v>0.1798963247727822</v>
       </c>
       <c r="AH51" t="n">
-        <v>0.2035724849641867</v>
+        <v>0.1798963247727822</v>
       </c>
       <c r="AI51" t="n">
-        <v>0.2035724849641867</v>
+        <v>0.1798963247727822</v>
       </c>
       <c r="AJ51" t="n">
-        <v>0.2035724849641867</v>
+        <v>0.1798963247727822</v>
       </c>
       <c r="AK51" t="n">
-        <v>0.2035724849641867</v>
+        <v>0.1798963247727822</v>
       </c>
       <c r="AL51" t="n">
-        <v>0.2035724849641867</v>
+        <v>0.1798963247727822</v>
       </c>
       <c r="AM51" t="n">
-        <v>0.1437071450395735</v>
+        <v>0.07363019854118745</v>
       </c>
       <c r="AN51" t="n">
-        <v>0.1437071450395735</v>
+        <v>0.07363019854118745</v>
       </c>
       <c r="AO51" t="n">
-        <v>0.1437071450395735</v>
+        <v>0.07363019854118745</v>
       </c>
     </row>
     <row r="52">
@@ -7076,25 +7076,25 @@
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="n">
-        <v>2.205882352941177</v>
+        <v>2.694411764705882</v>
       </c>
       <c r="G56" t="n">
         <v>0</v>
       </c>
       <c r="H56" t="n">
-        <v>0.3671547964358005</v>
+        <v>0.3684646262346155</v>
       </c>
       <c r="I56" t="n">
-        <v>0.039</v>
+        <v>0.03899999999999999</v>
       </c>
       <c r="J56" t="n">
-        <v>2.78</v>
+        <v>2.779999999999999</v>
       </c>
       <c r="K56" t="n">
-        <v>36.00000000000001</v>
+        <v>36</v>
       </c>
       <c r="L56" t="n">
-        <v>0.42</v>
+        <v>0.4199999999999999</v>
       </c>
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr"/>
@@ -7105,52 +7105,52 @@
         <v>0</v>
       </c>
       <c r="Q56" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="R56" t="n">
-        <v>0.039</v>
+        <v>0.03899999999999999</v>
       </c>
       <c r="S56" t="n">
-        <v>0.039</v>
+        <v>0.03899999999999999</v>
       </c>
       <c r="T56" t="n">
-        <v>0.039</v>
+        <v>0.03899999999999999</v>
       </c>
       <c r="U56" t="n">
-        <v>0.039</v>
+        <v>0.03899999999999999</v>
       </c>
       <c r="V56" t="n">
-        <v>0.039</v>
+        <v>0.03899999999999999</v>
       </c>
       <c r="W56" t="n">
-        <v>0.039</v>
+        <v>0.03899999999999999</v>
       </c>
       <c r="X56" t="n">
-        <v>0.039</v>
+        <v>0.03899999999999999</v>
       </c>
       <c r="Y56" t="n">
-        <v>0.039</v>
+        <v>0.03899999999999999</v>
       </c>
       <c r="Z56" t="n">
-        <v>0.039</v>
+        <v>0.03899999999999999</v>
       </c>
       <c r="AA56" t="n">
-        <v>0.039</v>
+        <v>0.03899999999999999</v>
       </c>
       <c r="AB56" t="n">
-        <v>0.039</v>
+        <v>0.03899999999999999</v>
       </c>
       <c r="AC56" t="n">
-        <v>0.039</v>
+        <v>0.03899999999999999</v>
       </c>
       <c r="AD56" t="n">
-        <v>0.0830769230769231</v>
+        <v>0.08307692307692306</v>
       </c>
       <c r="AE56" t="n">
-        <v>0.0830769230769231</v>
+        <v>0.08307692307692306</v>
       </c>
       <c r="AF56" t="n">
-        <v>0.0830769230769231</v>
+        <v>0.08307692307692306</v>
       </c>
       <c r="AG56" t="n">
         <v>0.1140983606557377</v>
@@ -7171,13 +7171,13 @@
         <v>0.1140983606557377</v>
       </c>
       <c r="AM56" t="n">
-        <v>0.0830769230769231</v>
+        <v>0.08307692307692306</v>
       </c>
       <c r="AN56" t="n">
-        <v>0.0830769230769231</v>
+        <v>0.08307692307692306</v>
       </c>
       <c r="AO56" t="n">
-        <v>0.0830769230769231</v>
+        <v>0.08307692307692306</v>
       </c>
     </row>
     <row r="57">
@@ -7552,13 +7552,13 @@
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="n">
-        <v>1.373313343328336</v>
+        <v>1.406296851574213</v>
       </c>
       <c r="G60" t="n">
         <v>0</v>
       </c>
       <c r="H60" t="n">
-        <v>0.3753487964221511</v>
+        <v>0.3749873699533331</v>
       </c>
       <c r="I60" t="n">
         <v>0.04730000000000001</v>
@@ -7581,7 +7581,7 @@
         <v>0</v>
       </c>
       <c r="Q60" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R60" t="n">
         <v>0.04730000000000001</v>
@@ -7671,19 +7671,19 @@
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="n">
-        <v>2.8834</v>
+        <v>3.08765</v>
       </c>
       <c r="G61" t="n">
         <v>0</v>
       </c>
       <c r="H61" t="n">
-        <v>0.4115443430009355</v>
+        <v>0.4117647098280165</v>
       </c>
       <c r="I61" t="n">
-        <v>0.04730000000000001</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="J61" t="n">
-        <v>3.67</v>
+        <v>3.670000000000001</v>
       </c>
       <c r="K61" t="n">
         <v>70</v>
@@ -7700,43 +7700,43 @@
         <v>0</v>
       </c>
       <c r="Q61" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="R61" t="n">
-        <v>0.04730000000000001</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="S61" t="n">
-        <v>0.04730000000000001</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="T61" t="n">
-        <v>0.04730000000000001</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="U61" t="n">
-        <v>0.04730000000000001</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="V61" t="n">
-        <v>0.04730000000000001</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="W61" t="n">
-        <v>0.04730000000000001</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="X61" t="n">
-        <v>0.04730000000000001</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="Y61" t="n">
-        <v>0.04730000000000001</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="Z61" t="n">
-        <v>0.04730000000000001</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="AA61" t="n">
-        <v>0.04730000000000001</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="AB61" t="n">
-        <v>0.04730000000000001</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="AC61" t="n">
-        <v>0.04730000000000001</v>
+        <v>0.04730000000000002</v>
       </c>
       <c r="AD61" t="n">
         <v>0.1769230769230769</v>
@@ -7790,25 +7790,25 @@
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="n">
-        <v>1.443956386292835</v>
+        <v>1.454330218068536</v>
       </c>
       <c r="G62" t="n">
         <v>0</v>
       </c>
       <c r="H62" t="n">
-        <v>0.3359219739647984</v>
+        <v>0.3357137921015227</v>
       </c>
       <c r="I62" t="n">
         <v>0.0473</v>
       </c>
       <c r="J62" t="n">
-        <v>3.67</v>
+        <v>3.669999999999999</v>
       </c>
       <c r="K62" t="n">
         <v>70</v>
       </c>
       <c r="L62" t="n">
-        <v>0.46</v>
+        <v>0.4600000000000001</v>
       </c>
       <c r="M62" t="inlineStr"/>
       <c r="N62" t="inlineStr"/>
@@ -7819,7 +7819,7 @@
         <v>0</v>
       </c>
       <c r="Q62" t="n">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="R62" t="n">
         <v>0.0473</v>
@@ -7858,13 +7858,13 @@
         <v>0.0473</v>
       </c>
       <c r="AD62" t="n">
-        <v>0.1769230769230769</v>
+        <v>0.176923076923077</v>
       </c>
       <c r="AE62" t="n">
-        <v>0.1769230769230769</v>
+        <v>0.176923076923077</v>
       </c>
       <c r="AF62" t="n">
-        <v>0.1769230769230769</v>
+        <v>0.176923076923077</v>
       </c>
       <c r="AG62" t="n">
         <v>0.2065573770491803</v>
@@ -7885,13 +7885,13 @@
         <v>0.2065573770491803</v>
       </c>
       <c r="AM62" t="n">
-        <v>0.1769230769230769</v>
+        <v>0.176923076923077</v>
       </c>
       <c r="AN62" t="n">
-        <v>0.1769230769230769</v>
+        <v>0.176923076923077</v>
       </c>
       <c r="AO62" t="n">
-        <v>0.1769230769230769</v>
+        <v>0.176923076923077</v>
       </c>
     </row>
     <row r="63">
@@ -8629,10 +8629,10 @@
         <v>0</v>
       </c>
       <c r="H69" t="n">
-        <v>0.324331100082713</v>
+        <v>0.3191022967553773</v>
       </c>
       <c r="I69" t="n">
-        <v>0.08265134776844894</v>
+        <v>0.08233720703759008</v>
       </c>
       <c r="J69" t="n">
         <v>1</v>
@@ -8652,43 +8652,43 @@
         <v>0</v>
       </c>
       <c r="Q69" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R69" t="n">
-        <v>0.08265134776844894</v>
+        <v>0.08233720703759008</v>
       </c>
       <c r="S69" t="n">
-        <v>0.08265134776844894</v>
+        <v>0.08233720703759008</v>
       </c>
       <c r="T69" t="n">
-        <v>0.08265134776844894</v>
+        <v>0.08233720703759008</v>
       </c>
       <c r="U69" t="n">
-        <v>0.08265134776844894</v>
+        <v>0.08233720703759008</v>
       </c>
       <c r="V69" t="n">
-        <v>0.08265134776844894</v>
+        <v>0.08233720703759008</v>
       </c>
       <c r="W69" t="n">
-        <v>0.08265134776844894</v>
+        <v>0.08233720703759008</v>
       </c>
       <c r="X69" t="n">
-        <v>0.08265134776844894</v>
+        <v>0.08233720703759008</v>
       </c>
       <c r="Y69" t="n">
-        <v>0.08265134776844894</v>
+        <v>0.08233720703759008</v>
       </c>
       <c r="Z69" t="n">
-        <v>0.08265134776844894</v>
+        <v>0.08233720703759008</v>
       </c>
       <c r="AA69" t="n">
-        <v>0.08265134776844894</v>
+        <v>0.08233720703759008</v>
       </c>
       <c r="AB69" t="n">
-        <v>0.08265134776844894</v>
+        <v>0.08233720703759008</v>
       </c>
       <c r="AC69" t="n">
-        <v>0.08265134776844894</v>
+        <v>0.08233720703759008</v>
       </c>
       <c r="AD69" t="n">
         <v>0.01071428571428571</v>
@@ -8700,22 +8700,22 @@
         <v>0.01071428571428571</v>
       </c>
       <c r="AG69" t="n">
-        <v>0.06038251366120219</v>
+        <v>0.06038251366120218</v>
       </c>
       <c r="AH69" t="n">
-        <v>0.06038251366120219</v>
+        <v>0.06038251366120218</v>
       </c>
       <c r="AI69" t="n">
-        <v>0.06038251366120219</v>
+        <v>0.06038251366120218</v>
       </c>
       <c r="AJ69" t="n">
-        <v>0.06038251366120219</v>
+        <v>0.06038251366120218</v>
       </c>
       <c r="AK69" t="n">
-        <v>0.06038251366120219</v>
+        <v>0.06038251366120218</v>
       </c>
       <c r="AL69" t="n">
-        <v>0.06038251366120219</v>
+        <v>0.06038251366120218</v>
       </c>
       <c r="AM69" t="n">
         <v>0.01071428571428571</v>
@@ -10051,16 +10051,16 @@
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="n">
-        <v>1.398</v>
+        <v>2.214</v>
       </c>
       <c r="G81" t="n">
         <v>0</v>
       </c>
       <c r="H81" t="n">
-        <v>0.3145135876042908</v>
+        <v>0.3456244587008821</v>
       </c>
       <c r="I81" t="n">
-        <v>0.1096732901203323</v>
+        <v>0.1116178005294899</v>
       </c>
       <c r="J81" t="n">
         <v>1</v>
@@ -10080,43 +10080,43 @@
         <v>0</v>
       </c>
       <c r="Q81" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R81" t="n">
-        <v>0.1096732901203323</v>
+        <v>0.1116178005294899</v>
       </c>
       <c r="S81" t="n">
-        <v>0.1096732901203323</v>
+        <v>0.1116178005294899</v>
       </c>
       <c r="T81" t="n">
-        <v>0.1096732901203323</v>
+        <v>0.1116178005294899</v>
       </c>
       <c r="U81" t="n">
-        <v>0.1096732901203323</v>
+        <v>0.1116178005294899</v>
       </c>
       <c r="V81" t="n">
-        <v>0.1096732901203323</v>
+        <v>0.1116178005294899</v>
       </c>
       <c r="W81" t="n">
-        <v>0.1096732901203323</v>
+        <v>0.1116178005294899</v>
       </c>
       <c r="X81" t="n">
-        <v>0.1096732901203323</v>
+        <v>0.1116178005294899</v>
       </c>
       <c r="Y81" t="n">
-        <v>0.1096732901203323</v>
+        <v>0.1116178005294899</v>
       </c>
       <c r="Z81" t="n">
-        <v>0.1096732901203323</v>
+        <v>0.1116178005294899</v>
       </c>
       <c r="AA81" t="n">
-        <v>0.1096732901203323</v>
+        <v>0.1116178005294899</v>
       </c>
       <c r="AB81" t="n">
-        <v>0.1096732901203323</v>
+        <v>0.1116178005294899</v>
       </c>
       <c r="AC81" t="n">
-        <v>0.1096732901203323</v>
+        <v>0.1116178005294899</v>
       </c>
       <c r="AD81" t="n">
         <v>0.01071428571428571</v>
@@ -10128,22 +10128,22 @@
         <v>0.01071428571428571</v>
       </c>
       <c r="AG81" t="n">
-        <v>0.06038251366120218</v>
+        <v>0.06038251366120219</v>
       </c>
       <c r="AH81" t="n">
-        <v>0.06038251366120218</v>
+        <v>0.06038251366120219</v>
       </c>
       <c r="AI81" t="n">
-        <v>0.06038251366120218</v>
+        <v>0.06038251366120219</v>
       </c>
       <c r="AJ81" t="n">
-        <v>0.06038251366120218</v>
+        <v>0.06038251366120219</v>
       </c>
       <c r="AK81" t="n">
-        <v>0.06038251366120218</v>
+        <v>0.06038251366120219</v>
       </c>
       <c r="AL81" t="n">
-        <v>0.06038251366120218</v>
+        <v>0.06038251366120219</v>
       </c>
       <c r="AM81" t="n">
         <v>0.01071428571428571</v>
@@ -11122,7 +11122,7 @@
       <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="n">
-        <v>22.80864672001289</v>
+        <v>23.53484398915174</v>
       </c>
       <c r="G90" t="n">
         <v>0</v>
@@ -11131,7 +11131,7 @@
         <v>0.4799999999999999</v>
       </c>
       <c r="I90" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="J90" t="n">
         <v>1</v>
@@ -11151,79 +11151,79 @@
         <v>1</v>
       </c>
       <c r="Q90" t="n">
-        <v>307</v>
+        <v>347</v>
       </c>
       <c r="R90" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="S90" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="T90" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="U90" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="V90" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="W90" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="X90" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="Y90" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="Z90" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="AA90" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="AB90" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="AC90" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="AD90" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AE90" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AF90" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AG90" t="n">
-        <v>0.1254098360655737</v>
+        <v>0.1254098360655738</v>
       </c>
       <c r="AH90" t="n">
-        <v>0.1254098360655737</v>
+        <v>0.1254098360655738</v>
       </c>
       <c r="AI90" t="n">
-        <v>0.1254098360655737</v>
+        <v>0.1254098360655738</v>
       </c>
       <c r="AJ90" t="n">
-        <v>0.1254098360655737</v>
+        <v>0.1254098360655738</v>
       </c>
       <c r="AK90" t="n">
-        <v>0.1254098360655737</v>
+        <v>0.1254098360655738</v>
       </c>
       <c r="AL90" t="n">
-        <v>0.1254098360655737</v>
+        <v>0.1254098360655738</v>
       </c>
       <c r="AM90" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AN90" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AO90" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
     </row>
     <row r="91">
@@ -11479,7 +11479,7 @@
       <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G93" t="n">
         <v>0</v>
@@ -11494,10 +11494,10 @@
         <v>2</v>
       </c>
       <c r="K93" t="n">
-        <v>135</v>
+        <v>97.5</v>
       </c>
       <c r="L93" t="n">
-        <v>0.075</v>
+        <v>0.0375</v>
       </c>
       <c r="M93" t="inlineStr"/>
       <c r="N93" t="inlineStr"/>
@@ -11508,7 +11508,7 @@
         <v>0</v>
       </c>
       <c r="Q93" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R93" t="n">
         <v>0.04</v>
@@ -11547,40 +11547,40 @@
         <v>0.04</v>
       </c>
       <c r="AD93" t="n">
-        <v>0.05563186813186814</v>
+        <v>0.02008928571428571</v>
       </c>
       <c r="AE93" t="n">
-        <v>0.05563186813186814</v>
+        <v>0.02008928571428571</v>
       </c>
       <c r="AF93" t="n">
-        <v>0.05563186813186814</v>
+        <v>0.02008928571428571</v>
       </c>
       <c r="AG93" t="n">
-        <v>0.6823770491803279</v>
+        <v>0.5128073770491803</v>
       </c>
       <c r="AH93" t="n">
-        <v>0.6823770491803279</v>
+        <v>0.5128073770491803</v>
       </c>
       <c r="AI93" t="n">
-        <v>0.6823770491803279</v>
+        <v>0.5128073770491803</v>
       </c>
       <c r="AJ93" t="n">
-        <v>0.6823770491803279</v>
+        <v>0.5128073770491803</v>
       </c>
       <c r="AK93" t="n">
-        <v>0.6823770491803279</v>
+        <v>0.5128073770491803</v>
       </c>
       <c r="AL93" t="n">
-        <v>0.6823770491803279</v>
+        <v>0.5128073770491803</v>
       </c>
       <c r="AM93" t="n">
-        <v>0.05563186813186814</v>
+        <v>0.02008928571428571</v>
       </c>
       <c r="AN93" t="n">
-        <v>0.05563186813186814</v>
+        <v>0.02008928571428571</v>
       </c>
       <c r="AO93" t="n">
-        <v>0.05563186813186814</v>
+        <v>0.02008928571428571</v>
       </c>
     </row>
     <row r="94">
@@ -12669,7 +12669,7 @@
       <c r="D103" t="inlineStr"/>
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="n">
-        <v>0.6186868686868687</v>
+        <v>1.237373737373737</v>
       </c>
       <c r="G103" t="n">
         <v>0</v>
@@ -12698,7 +12698,7 @@
         <v>0</v>
       </c>
       <c r="Q103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R103" t="n">
         <v>0.05</v>
@@ -12788,7 +12788,7 @@
       <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="n">
-        <v>3.898550724637681</v>
+        <v>4.347826086956522</v>
       </c>
       <c r="G104" t="n">
         <v>0</v>
@@ -12817,7 +12817,7 @@
         <v>0</v>
       </c>
       <c r="Q104" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R104" t="n">
         <v>0.05</v>
@@ -12913,10 +12913,10 @@
         <v>0</v>
       </c>
       <c r="H105" t="n">
-        <v>0.36</v>
+        <v>0.3599999999999999</v>
       </c>
       <c r="I105" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="J105" t="n">
         <v>1</v>
@@ -12936,43 +12936,43 @@
         <v>1</v>
       </c>
       <c r="Q105" t="n">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="R105" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="S105" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="T105" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="U105" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="V105" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="W105" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="X105" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="Y105" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="Z105" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="AA105" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="AB105" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="AC105" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="AD105" t="n">
         <v>0.02225274725274725</v>
@@ -13145,7 +13145,7 @@
       <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="n">
-        <v>24.83872727272727</v>
+        <v>25.20472727272728</v>
       </c>
       <c r="G107" t="n">
         <v>0</v>
@@ -13174,7 +13174,7 @@
         <v>1</v>
       </c>
       <c r="Q107" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="R107" t="n">
         <v>0</v>
@@ -13264,7 +13264,7 @@
       <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="n">
-        <v>0.6326530612244898</v>
+        <v>1.13265306122449</v>
       </c>
       <c r="G108" t="n">
         <v>0</v>
@@ -13293,7 +13293,7 @@
         <v>0</v>
       </c>
       <c r="Q108" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R108" t="n">
         <v>0.05</v>
@@ -14097,7 +14097,7 @@
       <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr"/>
       <c r="F115" t="n">
-        <v>0.2089951513124896</v>
+        <v>0.6269854539374686</v>
       </c>
       <c r="G115" t="n">
         <v>0</v>
@@ -14106,13 +14106,13 @@
         <v>0.35</v>
       </c>
       <c r="I115" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="J115" t="n">
         <v>1</v>
       </c>
       <c r="K115" t="n">
-        <v>7</v>
+        <v>7.000000000000001</v>
       </c>
       <c r="L115" t="n">
         <v>0.15</v>
@@ -14126,43 +14126,43 @@
         <v>0</v>
       </c>
       <c r="Q115" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R115" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="S115" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="T115" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="U115" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="V115" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="W115" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="X115" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="Y115" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="Z115" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="AA115" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="AB115" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="AC115" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="AD115" t="n">
         <v>0.00576923076923077</v>
@@ -14216,13 +14216,13 @@
       <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="n">
-        <v>0.1978925569496894</v>
+        <v>0.5936776708490681</v>
       </c>
       <c r="G116" t="n">
         <v>0</v>
       </c>
       <c r="H116" t="n">
-        <v>0.35</v>
+        <v>0.3499999999999999</v>
       </c>
       <c r="I116" t="n">
         <v>0.08</v>
@@ -14231,7 +14231,7 @@
         <v>1</v>
       </c>
       <c r="K116" t="n">
-        <v>7</v>
+        <v>6.999999999999999</v>
       </c>
       <c r="L116" t="n">
         <v>0.15</v>
@@ -14245,7 +14245,7 @@
         <v>1</v>
       </c>
       <c r="Q116" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R116" t="n">
         <v>0.08</v>
@@ -14284,40 +14284,40 @@
         <v>0.08</v>
       </c>
       <c r="AD116" t="n">
-        <v>0.00576923076923077</v>
+        <v>0.005769230769230769</v>
       </c>
       <c r="AE116" t="n">
-        <v>0.00576923076923077</v>
+        <v>0.005769230769230769</v>
       </c>
       <c r="AF116" t="n">
-        <v>0.00576923076923077</v>
+        <v>0.005769230769230769</v>
       </c>
       <c r="AG116" t="n">
-        <v>0.0325136612021858</v>
+        <v>0.03251366120218579</v>
       </c>
       <c r="AH116" t="n">
-        <v>0.0325136612021858</v>
+        <v>0.03251366120218579</v>
       </c>
       <c r="AI116" t="n">
-        <v>0.0325136612021858</v>
+        <v>0.03251366120218579</v>
       </c>
       <c r="AJ116" t="n">
-        <v>0.0325136612021858</v>
+        <v>0.03251366120218579</v>
       </c>
       <c r="AK116" t="n">
-        <v>0.0325136612021858</v>
+        <v>0.03251366120218579</v>
       </c>
       <c r="AL116" t="n">
-        <v>0.0325136612021858</v>
+        <v>0.03251366120218579</v>
       </c>
       <c r="AM116" t="n">
-        <v>0.00576923076923077</v>
+        <v>0.005769230769230769</v>
       </c>
       <c r="AN116" t="n">
-        <v>0.00576923076923077</v>
+        <v>0.005769230769230769</v>
       </c>
       <c r="AO116" t="n">
-        <v>0.00576923076923077</v>
+        <v>0.005769230769230769</v>
       </c>
     </row>
     <row r="117">
@@ -14335,7 +14335,7 @@
       <c r="D117" t="inlineStr"/>
       <c r="E117" t="inlineStr"/>
       <c r="F117" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G117" t="n">
         <v>0</v>
@@ -14364,7 +14364,7 @@
         <v>0</v>
       </c>
       <c r="Q117" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R117" t="n">
         <v>0.08</v>
@@ -14454,13 +14454,13 @@
       <c r="D118" t="inlineStr"/>
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="n">
-        <v>0.7542857142857142</v>
+        <v>1.154285714285714</v>
       </c>
       <c r="G118" t="n">
         <v>0</v>
       </c>
       <c r="H118" t="n">
-        <v>0.5600000000000002</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I118" t="n">
         <v>0.05</v>
@@ -14483,7 +14483,7 @@
         <v>0</v>
       </c>
       <c r="Q118" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R118" t="n">
         <v>0.05</v>
@@ -14692,7 +14692,7 @@
       <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="n">
-        <v>0.6257575757575757</v>
+        <v>0.6919191919191919</v>
       </c>
       <c r="G120" t="n">
         <v>0</v>
@@ -14701,7 +14701,7 @@
         <v>0.36</v>
       </c>
       <c r="I120" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="J120" t="n">
         <v>1</v>
@@ -14721,52 +14721,52 @@
         <v>0</v>
       </c>
       <c r="Q120" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R120" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="S120" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="T120" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="U120" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="V120" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="W120" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="X120" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="Y120" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="Z120" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="AA120" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="AB120" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="AC120" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="AD120" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AE120" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AF120" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AG120" t="n">
         <v>0.1254098360655738</v>
@@ -14787,13 +14787,13 @@
         <v>0.1254098360655738</v>
       </c>
       <c r="AM120" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AN120" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AO120" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
     </row>
     <row r="121">
@@ -15763,7 +15763,7 @@
       <c r="D129" t="inlineStr"/>
       <c r="E129" t="inlineStr"/>
       <c r="F129" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="G129" t="n">
         <v>0</v>
@@ -15792,7 +15792,7 @@
         <v>0</v>
       </c>
       <c r="Q129" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R129" t="n">
         <v>0.075</v>
@@ -16120,7 +16120,7 @@
       <c r="D132" t="inlineStr"/>
       <c r="E132" t="inlineStr"/>
       <c r="F132" t="n">
-        <v>1.333333333333333</v>
+        <v>2.666666666666667</v>
       </c>
       <c r="G132" t="n">
         <v>0</v>
@@ -16149,7 +16149,7 @@
         <v>0</v>
       </c>
       <c r="Q132" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="R132" t="n">
         <v>0.05</v>
@@ -17191,22 +17191,22 @@
       <c r="D141" t="inlineStr"/>
       <c r="E141" t="inlineStr"/>
       <c r="F141" t="n">
-        <v>0.9355999999999999</v>
+        <v>2.839999999999999</v>
       </c>
       <c r="G141" t="n">
         <v>0</v>
       </c>
       <c r="H141" t="n">
-        <v>0.4463847399676085</v>
+        <v>0.4692988084326307</v>
       </c>
       <c r="I141" t="n">
-        <v>0.03995627136944394</v>
+        <v>0.04719786892758936</v>
       </c>
       <c r="J141" t="n">
         <v>1</v>
       </c>
       <c r="K141" t="n">
-        <v>17.40093575670326</v>
+        <v>17.5627864344638</v>
       </c>
       <c r="L141" t="n">
         <v>0.15</v>
@@ -17220,79 +17220,79 @@
         <v>0</v>
       </c>
       <c r="Q141" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="R141" t="n">
-        <v>0.03995627136944394</v>
+        <v>0.04719786892758936</v>
       </c>
       <c r="S141" t="n">
-        <v>0.03995627136944394</v>
+        <v>0.04719786892758936</v>
       </c>
       <c r="T141" t="n">
-        <v>0.03995627136944394</v>
+        <v>0.04719786892758936</v>
       </c>
       <c r="U141" t="n">
-        <v>0.03995627136944394</v>
+        <v>0.04719786892758936</v>
       </c>
       <c r="V141" t="n">
-        <v>0.03995627136944394</v>
+        <v>0.04719786892758936</v>
       </c>
       <c r="W141" t="n">
-        <v>0.03995627136944394</v>
+        <v>0.04719786892758936</v>
       </c>
       <c r="X141" t="n">
-        <v>0.03995627136944394</v>
+        <v>0.04719786892758936</v>
       </c>
       <c r="Y141" t="n">
-        <v>0.03995627136944394</v>
+        <v>0.04719786892758936</v>
       </c>
       <c r="Z141" t="n">
-        <v>0.03995627136944394</v>
+        <v>0.04719786892758936</v>
       </c>
       <c r="AA141" t="n">
-        <v>0.03995627136944394</v>
+        <v>0.04719786892758936</v>
       </c>
       <c r="AB141" t="n">
-        <v>0.03995627136944394</v>
+        <v>0.04719786892758936</v>
       </c>
       <c r="AC141" t="n">
-        <v>0.03995627136944394</v>
+        <v>0.04719786892758936</v>
       </c>
       <c r="AD141" t="n">
-        <v>0.01434143056871148</v>
+        <v>0.01447482398444818</v>
       </c>
       <c r="AE141" t="n">
-        <v>0.01434143056871148</v>
+        <v>0.01447482398444818</v>
       </c>
       <c r="AF141" t="n">
-        <v>0.01434143056871148</v>
+        <v>0.01447482398444818</v>
       </c>
       <c r="AG141" t="n">
-        <v>0.08082401854206432</v>
+        <v>0.08157578398521435</v>
       </c>
       <c r="AH141" t="n">
-        <v>0.08082401854206432</v>
+        <v>0.08157578398521435</v>
       </c>
       <c r="AI141" t="n">
-        <v>0.08082401854206432</v>
+        <v>0.08157578398521435</v>
       </c>
       <c r="AJ141" t="n">
-        <v>0.08082401854206432</v>
+        <v>0.08157578398521435</v>
       </c>
       <c r="AK141" t="n">
-        <v>0.08082401854206432</v>
+        <v>0.08157578398521435</v>
       </c>
       <c r="AL141" t="n">
-        <v>0.08082401854206432</v>
+        <v>0.08157578398521435</v>
       </c>
       <c r="AM141" t="n">
-        <v>0.01434143056871148</v>
+        <v>0.01447482398444818</v>
       </c>
       <c r="AN141" t="n">
-        <v>0.01434143056871148</v>
+        <v>0.01447482398444818</v>
       </c>
       <c r="AO141" t="n">
-        <v>0.01434143056871148</v>
+        <v>0.01447482398444818</v>
       </c>
     </row>
     <row r="142">
@@ -17667,7 +17667,7 @@
       <c r="D145" t="inlineStr"/>
       <c r="E145" t="inlineStr"/>
       <c r="F145" t="n">
-        <v>0.2589285714285715</v>
+        <v>0.5178571428571429</v>
       </c>
       <c r="G145" t="n">
         <v>0</v>
@@ -17696,7 +17696,7 @@
         <v>1</v>
       </c>
       <c r="Q145" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R145" t="n">
         <v>0.05</v>
@@ -19214,7 +19214,7 @@
       <c r="D158" t="inlineStr"/>
       <c r="E158" t="inlineStr"/>
       <c r="F158" t="n">
-        <v>0.5434179357021997</v>
+        <v>0.8479864636209813</v>
       </c>
       <c r="G158" t="n">
         <v>0</v>
@@ -19243,7 +19243,7 @@
         <v>1</v>
       </c>
       <c r="Q158" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R158" t="n">
         <v>0.05</v>
@@ -19333,7 +19333,7 @@
       <c r="D159" t="inlineStr"/>
       <c r="E159" t="inlineStr"/>
       <c r="F159" t="n">
-        <v>0.8668354430379747</v>
+        <v>0.9235443037974682</v>
       </c>
       <c r="G159" t="n">
         <v>0</v>
@@ -19342,13 +19342,13 @@
         <v>0.51</v>
       </c>
       <c r="I159" t="n">
-        <v>0.05</v>
+        <v>0.04999999999999999</v>
       </c>
       <c r="J159" t="n">
         <v>1</v>
       </c>
       <c r="K159" t="n">
-        <v>26.05769230769231</v>
+        <v>25.23423423423423</v>
       </c>
       <c r="L159" t="n">
         <v>0.15</v>
@@ -19362,79 +19362,79 @@
         <v>1</v>
       </c>
       <c r="Q159" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R159" t="n">
-        <v>0.05</v>
+        <v>0.04999999999999999</v>
       </c>
       <c r="S159" t="n">
-        <v>0.05</v>
+        <v>0.04999999999999999</v>
       </c>
       <c r="T159" t="n">
-        <v>0.05</v>
+        <v>0.04999999999999999</v>
       </c>
       <c r="U159" t="n">
-        <v>0.05</v>
+        <v>0.04999999999999999</v>
       </c>
       <c r="V159" t="n">
-        <v>0.05</v>
+        <v>0.04999999999999999</v>
       </c>
       <c r="W159" t="n">
-        <v>0.05</v>
+        <v>0.04999999999999999</v>
       </c>
       <c r="X159" t="n">
-        <v>0.05</v>
+        <v>0.04999999999999999</v>
       </c>
       <c r="Y159" t="n">
-        <v>0.05</v>
+        <v>0.04999999999999999</v>
       </c>
       <c r="Z159" t="n">
-        <v>0.05</v>
+        <v>0.04999999999999999</v>
       </c>
       <c r="AA159" t="n">
-        <v>0.05</v>
+        <v>0.04999999999999999</v>
       </c>
       <c r="AB159" t="n">
-        <v>0.05</v>
+        <v>0.04999999999999999</v>
       </c>
       <c r="AC159" t="n">
-        <v>0.05</v>
+        <v>0.04999999999999999</v>
       </c>
       <c r="AD159" t="n">
-        <v>0.02147612003381235</v>
+        <v>0.0207974457974458</v>
       </c>
       <c r="AE159" t="n">
-        <v>0.02147612003381235</v>
+        <v>0.0207974457974458</v>
       </c>
       <c r="AF159" t="n">
-        <v>0.02147612003381235</v>
+        <v>0.0207974457974458</v>
       </c>
       <c r="AG159" t="n">
-        <v>0.1210329970575872</v>
+        <v>0.1172081917983557</v>
       </c>
       <c r="AH159" t="n">
-        <v>0.1210329970575872</v>
+        <v>0.1172081917983557</v>
       </c>
       <c r="AI159" t="n">
-        <v>0.1210329970575872</v>
+        <v>0.1172081917983557</v>
       </c>
       <c r="AJ159" t="n">
-        <v>0.1210329970575872</v>
+        <v>0.1172081917983557</v>
       </c>
       <c r="AK159" t="n">
-        <v>0.1210329970575872</v>
+        <v>0.1172081917983557</v>
       </c>
       <c r="AL159" t="n">
-        <v>0.1210329970575872</v>
+        <v>0.1172081917983557</v>
       </c>
       <c r="AM159" t="n">
-        <v>0.02147612003381235</v>
+        <v>0.0207974457974458</v>
       </c>
       <c r="AN159" t="n">
-        <v>0.02147612003381235</v>
+        <v>0.0207974457974458</v>
       </c>
       <c r="AO159" t="n">
-        <v>0.02147612003381235</v>
+        <v>0.0207974457974458</v>
       </c>
     </row>
     <row r="160">
@@ -19690,22 +19690,22 @@
       <c r="D162" t="inlineStr"/>
       <c r="E162" t="inlineStr"/>
       <c r="F162" t="n">
-        <v>6.729264392324094</v>
+        <v>7.059754797441364</v>
       </c>
       <c r="G162" t="n">
         <v>0</v>
       </c>
       <c r="H162" t="n">
-        <v>0.48</v>
+        <v>0.4799999999999999</v>
       </c>
       <c r="I162" t="n">
-        <v>0.0593739253387771</v>
+        <v>0.05898604536714707</v>
       </c>
       <c r="J162" t="n">
         <v>1</v>
       </c>
       <c r="K162" t="n">
-        <v>26.51317675205087</v>
+        <v>26.53332081985374</v>
       </c>
       <c r="L162" t="n">
         <v>0.15</v>
@@ -19719,79 +19719,79 @@
         <v>1</v>
       </c>
       <c r="Q162" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="R162" t="n">
-        <v>0.0593739253387771</v>
+        <v>0.05898604536714707</v>
       </c>
       <c r="S162" t="n">
-        <v>0.0593739253387771</v>
+        <v>0.05898604536714707</v>
       </c>
       <c r="T162" t="n">
-        <v>0.0593739253387771</v>
+        <v>0.05898604536714707</v>
       </c>
       <c r="U162" t="n">
-        <v>0.0593739253387771</v>
+        <v>0.05898604536714707</v>
       </c>
       <c r="V162" t="n">
-        <v>0.0593739253387771</v>
+        <v>0.05898604536714707</v>
       </c>
       <c r="W162" t="n">
-        <v>0.0593739253387771</v>
+        <v>0.05898604536714707</v>
       </c>
       <c r="X162" t="n">
-        <v>0.0593739253387771</v>
+        <v>0.05898604536714707</v>
       </c>
       <c r="Y162" t="n">
-        <v>0.0593739253387771</v>
+        <v>0.05898604536714707</v>
       </c>
       <c r="Z162" t="n">
-        <v>0.0593739253387771</v>
+        <v>0.05898604536714707</v>
       </c>
       <c r="AA162" t="n">
-        <v>0.0593739253387771</v>
+        <v>0.05898604536714707</v>
       </c>
       <c r="AB162" t="n">
-        <v>0.0593739253387771</v>
+        <v>0.05898604536714707</v>
       </c>
       <c r="AC162" t="n">
-        <v>0.0593739253387771</v>
+        <v>0.05898604536714707</v>
       </c>
       <c r="AD162" t="n">
-        <v>0.02185151930114083</v>
+        <v>0.02186812155482451</v>
       </c>
       <c r="AE162" t="n">
-        <v>0.02185151930114083</v>
+        <v>0.02186812155482451</v>
       </c>
       <c r="AF162" t="n">
-        <v>0.02185151930114083</v>
+        <v>0.02186812155482451</v>
       </c>
       <c r="AG162" t="n">
-        <v>0.1231486351871215</v>
+        <v>0.1232422005293753</v>
       </c>
       <c r="AH162" t="n">
-        <v>0.1231486351871215</v>
+        <v>0.1232422005293753</v>
       </c>
       <c r="AI162" t="n">
-        <v>0.1231486351871215</v>
+        <v>0.1232422005293753</v>
       </c>
       <c r="AJ162" t="n">
-        <v>0.1231486351871215</v>
+        <v>0.1232422005293753</v>
       </c>
       <c r="AK162" t="n">
-        <v>0.1231486351871215</v>
+        <v>0.1232422005293753</v>
       </c>
       <c r="AL162" t="n">
-        <v>0.1231486351871215</v>
+        <v>0.1232422005293753</v>
       </c>
       <c r="AM162" t="n">
-        <v>0.02185151930114083</v>
+        <v>0.02186812155482451</v>
       </c>
       <c r="AN162" t="n">
-        <v>0.02185151930114083</v>
+        <v>0.02186812155482451</v>
       </c>
       <c r="AO162" t="n">
-        <v>0.02185151930114083</v>
+        <v>0.02186812155482451</v>
       </c>
     </row>
     <row r="163">
@@ -20761,7 +20761,7 @@
       <c r="D171" t="inlineStr"/>
       <c r="E171" t="inlineStr"/>
       <c r="F171" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G171" t="n">
         <v>0</v>
@@ -20790,7 +20790,7 @@
         <v>1</v>
       </c>
       <c r="Q171" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R171" t="n">
         <v>0.08000000000000002</v>
@@ -21118,7 +21118,7 @@
       <c r="D174" t="inlineStr"/>
       <c r="E174" t="inlineStr"/>
       <c r="F174" t="n">
-        <v>0.6915322580645161</v>
+        <v>1.377016129032258</v>
       </c>
       <c r="G174" t="n">
         <v>0</v>
@@ -21147,7 +21147,7 @@
         <v>1</v>
       </c>
       <c r="Q174" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R174" t="n">
         <v>0.08</v>
@@ -21951,7 +21951,7 @@
       <c r="D181" t="inlineStr"/>
       <c r="E181" t="inlineStr"/>
       <c r="F181" t="n">
-        <v>0.7993333333333333</v>
+        <v>1.399333333333333</v>
       </c>
       <c r="G181" t="n">
         <v>0</v>
@@ -21980,7 +21980,7 @@
         <v>1</v>
       </c>
       <c r="Q181" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R181" t="n">
         <v>0.05</v>
@@ -22070,7 +22070,7 @@
       <c r="D182" t="inlineStr"/>
       <c r="E182" t="inlineStr"/>
       <c r="F182" t="n">
-        <v>1.369622641509434</v>
+        <v>2.077169811320755</v>
       </c>
       <c r="G182" t="n">
         <v>0</v>
@@ -22099,7 +22099,7 @@
         <v>1</v>
       </c>
       <c r="Q182" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R182" t="n">
         <v>0.08</v>
@@ -22546,7 +22546,7 @@
       <c r="D186" t="inlineStr"/>
       <c r="E186" t="inlineStr"/>
       <c r="F186" t="n">
-        <v>1.261818181818182</v>
+        <v>1.283636363636364</v>
       </c>
       <c r="G186" t="n">
         <v>0</v>
@@ -22575,7 +22575,7 @@
         <v>0</v>
       </c>
       <c r="Q186" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R186" t="n">
         <v>0.05</v>
@@ -23260,7 +23260,7 @@
       <c r="D192" t="inlineStr"/>
       <c r="E192" t="inlineStr"/>
       <c r="F192" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G192" t="n">
         <v>0</v>
@@ -23289,7 +23289,7 @@
         <v>0</v>
       </c>
       <c r="Q192" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="R192" t="n">
         <v>0.08</v>
@@ -23379,7 +23379,7 @@
       <c r="D193" t="inlineStr"/>
       <c r="E193" t="inlineStr"/>
       <c r="F193" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="G193" t="n">
         <v>0</v>
@@ -23408,7 +23408,7 @@
         <v>0</v>
       </c>
       <c r="Q193" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R193" t="n">
         <v>0.08</v>
@@ -24093,13 +24093,13 @@
       <c r="D199" t="inlineStr"/>
       <c r="E199" t="inlineStr"/>
       <c r="F199" t="n">
-        <v>1.679056748466258</v>
+        <v>1.990253067484663</v>
       </c>
       <c r="G199" t="n">
         <v>0</v>
       </c>
       <c r="H199" t="n">
-        <v>0.5759713435057684</v>
+        <v>0.5750784593437946</v>
       </c>
       <c r="I199" t="n">
         <v>0.05</v>
@@ -24122,7 +24122,7 @@
         <v>0</v>
       </c>
       <c r="Q199" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="R199" t="n">
         <v>0.05</v>
@@ -24212,7 +24212,7 @@
       <c r="D200" t="inlineStr"/>
       <c r="E200" t="inlineStr"/>
       <c r="F200" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="G200" t="n">
         <v>0</v>
@@ -24241,7 +24241,7 @@
         <v>0</v>
       </c>
       <c r="Q200" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R200" t="n">
         <v>0.075</v>
@@ -26235,7 +26235,7 @@
       <c r="D217" t="inlineStr"/>
       <c r="E217" t="inlineStr"/>
       <c r="F217" t="n">
-        <v>2.254241338112306</v>
+        <v>3.659737156511351</v>
       </c>
       <c r="G217" t="n">
         <v>0</v>
@@ -26244,7 +26244,7 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="I217" t="n">
-        <v>0.05</v>
+        <v>0.05000000000000001</v>
       </c>
       <c r="J217" t="n">
         <v>1</v>
@@ -26264,43 +26264,43 @@
         <v>0</v>
       </c>
       <c r="Q217" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="R217" t="n">
-        <v>0.05</v>
+        <v>0.05000000000000001</v>
       </c>
       <c r="S217" t="n">
-        <v>0.05</v>
+        <v>0.05000000000000001</v>
       </c>
       <c r="T217" t="n">
-        <v>0.05</v>
+        <v>0.05000000000000001</v>
       </c>
       <c r="U217" t="n">
-        <v>0.05</v>
+        <v>0.05000000000000001</v>
       </c>
       <c r="V217" t="n">
-        <v>0.05</v>
+        <v>0.05000000000000001</v>
       </c>
       <c r="W217" t="n">
-        <v>0.05</v>
+        <v>0.05000000000000001</v>
       </c>
       <c r="X217" t="n">
-        <v>0.05</v>
+        <v>0.05000000000000001</v>
       </c>
       <c r="Y217" t="n">
-        <v>0.05</v>
+        <v>0.05000000000000001</v>
       </c>
       <c r="Z217" t="n">
-        <v>0.05</v>
+        <v>0.05000000000000001</v>
       </c>
       <c r="AA217" t="n">
-        <v>0.05</v>
+        <v>0.05000000000000001</v>
       </c>
       <c r="AB217" t="n">
-        <v>0.05</v>
+        <v>0.05000000000000001</v>
       </c>
       <c r="AC217" t="n">
-        <v>0.05</v>
+        <v>0.05000000000000001</v>
       </c>
       <c r="AD217" t="n">
         <v>0.02225274725274725</v>
@@ -27425,7 +27425,7 @@
       <c r="D227" t="inlineStr"/>
       <c r="E227" t="inlineStr"/>
       <c r="F227" t="n">
-        <v>0.4803252032520325</v>
+        <v>0.8632520325203252</v>
       </c>
       <c r="G227" t="n">
         <v>0</v>
@@ -27434,7 +27434,7 @@
         <v>0.6</v>
       </c>
       <c r="I227" t="n">
-        <v>0.009999999999999998</v>
+        <v>0.01</v>
       </c>
       <c r="J227" t="n">
         <v>1</v>
@@ -27454,43 +27454,43 @@
         <v>0</v>
       </c>
       <c r="Q227" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R227" t="n">
-        <v>0.009999999999999998</v>
+        <v>0.01</v>
       </c>
       <c r="S227" t="n">
-        <v>0.009999999999999998</v>
+        <v>0.01</v>
       </c>
       <c r="T227" t="n">
-        <v>0.009999999999999998</v>
+        <v>0.01</v>
       </c>
       <c r="U227" t="n">
-        <v>0.009999999999999998</v>
+        <v>0.01</v>
       </c>
       <c r="V227" t="n">
-        <v>0.009999999999999998</v>
+        <v>0.01</v>
       </c>
       <c r="W227" t="n">
-        <v>0.009999999999999998</v>
+        <v>0.01</v>
       </c>
       <c r="X227" t="n">
-        <v>0.009999999999999998</v>
+        <v>0.01</v>
       </c>
       <c r="Y227" t="n">
-        <v>0.009999999999999998</v>
+        <v>0.01</v>
       </c>
       <c r="Z227" t="n">
-        <v>0.009999999999999998</v>
+        <v>0.01</v>
       </c>
       <c r="AA227" t="n">
-        <v>0.009999999999999998</v>
+        <v>0.01</v>
       </c>
       <c r="AB227" t="n">
-        <v>0.009999999999999998</v>
+        <v>0.01</v>
       </c>
       <c r="AC227" t="n">
-        <v>0.009999999999999998</v>
+        <v>0.01</v>
       </c>
       <c r="AD227" t="n">
         <v>0</v>
@@ -28020,7 +28020,7 @@
       <c r="D232" t="inlineStr"/>
       <c r="E232" t="inlineStr"/>
       <c r="F232" t="n">
-        <v>0.46</v>
+        <v>0.5171428571428572</v>
       </c>
       <c r="G232" t="n">
         <v>0</v>
@@ -28049,7 +28049,7 @@
         <v>0</v>
       </c>
       <c r="Q232" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R232" t="n">
         <v>0.05</v>
@@ -28139,7 +28139,7 @@
       <c r="D233" t="inlineStr"/>
       <c r="E233" t="inlineStr"/>
       <c r="F233" t="n">
-        <v>1.364714285714286</v>
+        <v>1.994571428571429</v>
       </c>
       <c r="G233" t="n">
         <v>0</v>
@@ -28168,7 +28168,7 @@
         <v>0</v>
       </c>
       <c r="Q233" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="R233" t="n">
         <v>0.05</v>
@@ -28496,16 +28496,16 @@
       <c r="D236" t="inlineStr"/>
       <c r="E236" t="inlineStr"/>
       <c r="F236" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.08928571428571429</v>
       </c>
       <c r="G236" t="n">
         <v>0</v>
       </c>
       <c r="H236" t="n">
-        <v>0.5178947368421053</v>
+        <v>0.5483443708609272</v>
       </c>
       <c r="I236" t="n">
-        <v>0.03546342490562927</v>
+        <v>0.04085447262274689</v>
       </c>
       <c r="J236" t="n">
         <v>1</v>
@@ -28525,43 +28525,43 @@
         <v>0</v>
       </c>
       <c r="Q236" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R236" t="n">
-        <v>0.03546342490562927</v>
+        <v>0.04085447262274689</v>
       </c>
       <c r="S236" t="n">
-        <v>0.03546342490562927</v>
+        <v>0.04085447262274689</v>
       </c>
       <c r="T236" t="n">
-        <v>0.03546342490562927</v>
+        <v>0.04085447262274689</v>
       </c>
       <c r="U236" t="n">
-        <v>0.03546342490562927</v>
+        <v>0.04085447262274689</v>
       </c>
       <c r="V236" t="n">
-        <v>0.03546342490562927</v>
+        <v>0.04085447262274689</v>
       </c>
       <c r="W236" t="n">
-        <v>0.03546342490562927</v>
+        <v>0.04085447262274689</v>
       </c>
       <c r="X236" t="n">
-        <v>0.03546342490562927</v>
+        <v>0.04085447262274689</v>
       </c>
       <c r="Y236" t="n">
-        <v>0.03546342490562927</v>
+        <v>0.04085447262274689</v>
       </c>
       <c r="Z236" t="n">
-        <v>0.03546342490562927</v>
+        <v>0.04085447262274689</v>
       </c>
       <c r="AA236" t="n">
-        <v>0.03546342490562927</v>
+        <v>0.04085447262274689</v>
       </c>
       <c r="AB236" t="n">
-        <v>0.03546342490562927</v>
+        <v>0.04085447262274689</v>
       </c>
       <c r="AC236" t="n">
-        <v>0.03546342490562927</v>
+        <v>0.04085447262274689</v>
       </c>
       <c r="AD236" t="n">
         <v>0.02225274725274725</v>
@@ -30995,13 +30995,13 @@
       <c r="D257" t="inlineStr"/>
       <c r="E257" t="inlineStr"/>
       <c r="F257" t="n">
-        <v>2.373670886075949</v>
+        <v>33.36101265822784</v>
       </c>
       <c r="G257" t="n">
         <v>0</v>
       </c>
       <c r="H257" t="n">
-        <v>0.5600000000000002</v>
+        <v>0.5599999999999999</v>
       </c>
       <c r="I257" t="n">
         <v>0.05</v>
@@ -31024,7 +31024,7 @@
         <v>0</v>
       </c>
       <c r="Q257" t="n">
-        <v>7</v>
+        <v>97</v>
       </c>
       <c r="R257" t="n">
         <v>0.05</v>
@@ -31114,16 +31114,16 @@
       <c r="D258" t="inlineStr"/>
       <c r="E258" t="inlineStr"/>
       <c r="F258" t="n">
-        <v>0.9579356568364612</v>
+        <v>3.528981233243969</v>
       </c>
       <c r="G258" t="n">
         <v>0</v>
       </c>
       <c r="H258" t="n">
-        <v>0.3599999999999999</v>
+        <v>0.3600000000000001</v>
       </c>
       <c r="I258" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000003</v>
       </c>
       <c r="J258" t="n">
         <v>1</v>
@@ -31143,52 +31143,52 @@
         <v>0</v>
       </c>
       <c r="Q258" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="R258" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000003</v>
       </c>
       <c r="S258" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000003</v>
       </c>
       <c r="T258" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000003</v>
       </c>
       <c r="U258" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000003</v>
       </c>
       <c r="V258" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000003</v>
       </c>
       <c r="W258" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000003</v>
       </c>
       <c r="X258" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000003</v>
       </c>
       <c r="Y258" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000003</v>
       </c>
       <c r="Z258" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000003</v>
       </c>
       <c r="AA258" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000003</v>
       </c>
       <c r="AB258" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000003</v>
       </c>
       <c r="AC258" t="n">
-        <v>0.08</v>
+        <v>0.08000000000000003</v>
       </c>
       <c r="AD258" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AE258" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AF258" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AG258" t="n">
         <v>0.1254098360655738</v>
@@ -31209,13 +31209,13 @@
         <v>0.1254098360655738</v>
       </c>
       <c r="AM258" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AN258" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AO258" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
     </row>
     <row r="259">
@@ -31233,7 +31233,7 @@
       <c r="D259" t="inlineStr"/>
       <c r="E259" t="inlineStr"/>
       <c r="F259" t="n">
-        <v>0.8068836045056321</v>
+        <v>5.028827701293284</v>
       </c>
       <c r="G259" t="n">
         <v>0</v>
@@ -31262,7 +31262,7 @@
         <v>0</v>
       </c>
       <c r="Q259" t="n">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="R259" t="n">
         <v>0.08</v>
@@ -31301,13 +31301,13 @@
         <v>0.08</v>
       </c>
       <c r="AD259" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AE259" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AF259" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AG259" t="n">
         <v>0.1254098360655738</v>
@@ -31328,13 +31328,13 @@
         <v>0.1254098360655738</v>
       </c>
       <c r="AM259" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AN259" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
       <c r="AO259" t="n">
-        <v>0.02225274725274725</v>
+        <v>0.02225274725274726</v>
       </c>
     </row>
     <row r="260">
@@ -31590,7 +31590,7 @@
       <c r="D262" t="inlineStr"/>
       <c r="E262" t="inlineStr"/>
       <c r="F262" t="n">
-        <v>0.6715447154471544</v>
+        <v>0.943089430894309</v>
       </c>
       <c r="G262" t="n">
         <v>0</v>
@@ -31619,7 +31619,7 @@
         <v>0</v>
       </c>
       <c r="Q262" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R262" t="n">
         <v>0.05</v>
@@ -31709,16 +31709,16 @@
       <c r="D263" t="inlineStr"/>
       <c r="E263" t="inlineStr"/>
       <c r="F263" t="n">
-        <v>1.857798165137615</v>
+        <v>8.669724770642201</v>
       </c>
       <c r="G263" t="n">
         <v>0</v>
       </c>
       <c r="H263" t="n">
-        <v>0.35</v>
+        <v>0.3499999999999999</v>
       </c>
       <c r="I263" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="J263" t="n">
         <v>1</v>
@@ -31738,43 +31738,43 @@
         <v>0</v>
       </c>
       <c r="Q263" t="n">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="R263" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="S263" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="T263" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="U263" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="V263" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="W263" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="X263" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="Y263" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="Z263" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="AA263" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="AB263" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="AC263" t="n">
-        <v>0.08</v>
+        <v>0.07999999999999999</v>
       </c>
       <c r="AD263" t="n">
         <v>0.01071428571428571</v>
@@ -32066,7 +32066,7 @@
       <c r="D266" t="inlineStr"/>
       <c r="E266" t="inlineStr"/>
       <c r="F266" t="n">
-        <v>0.7721518987341772</v>
+        <v>1.10126582278481</v>
       </c>
       <c r="G266" t="n">
         <v>0</v>
@@ -32095,7 +32095,7 @@
         <v>0</v>
       </c>
       <c r="Q266" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="R266" t="n">
         <v>0.089</v>
@@ -32143,22 +32143,22 @@
         <v>0.01730769230769231</v>
       </c>
       <c r="AG266" t="n">
-        <v>0.09754098360655739</v>
+        <v>0.09754098360655737</v>
       </c>
       <c r="AH266" t="n">
-        <v>0.09754098360655739</v>
+        <v>0.09754098360655737</v>
       </c>
       <c r="AI266" t="n">
-        <v>0.09754098360655739</v>
+        <v>0.09754098360655737</v>
       </c>
       <c r="AJ266" t="n">
-        <v>0.09754098360655739</v>
+        <v>0.09754098360655737</v>
       </c>
       <c r="AK266" t="n">
-        <v>0.09754098360655739</v>
+        <v>0.09754098360655737</v>
       </c>
       <c r="AL266" t="n">
-        <v>0.09754098360655739</v>
+        <v>0.09754098360655737</v>
       </c>
       <c r="AM266" t="n">
         <v>0.01730769230769231</v>
@@ -32304,7 +32304,7 @@
       <c r="D268" t="inlineStr"/>
       <c r="E268" t="inlineStr"/>
       <c r="F268" t="n">
-        <v>0.4114285714285714</v>
+        <v>0.8228571428571428</v>
       </c>
       <c r="G268" t="n">
         <v>0</v>
@@ -32333,7 +32333,7 @@
         <v>0</v>
       </c>
       <c r="Q268" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R268" t="n">
         <v>0.089</v>

</xml_diff>